<commit_message>
Update live Hitter Tool data
</commit_message>
<xml_diff>
--- a/outputs/daily/hr_rankings_2026-09-16.xlsx
+++ b/outputs/daily/hr_rankings_2026-09-16.xlsx
@@ -2444,7 +2444,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -5820,7 +5820,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -6936,7 +6936,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -10300,7 +10300,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -10580,7 +10580,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -10860,7 +10860,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -11976,7 +11976,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -13376,7 +13376,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -13656,7 +13656,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -14496,7 +14496,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -15336,7 +15336,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -17576,7 +17576,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -19252,7 +19252,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -20652,7 +20652,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -20932,7 +20932,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -23456,7 +23456,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -25700,7 +25700,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -27104,7 +27104,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -27948,7 +27948,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -28228,7 +28228,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -28508,7 +28508,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -30748,7 +30748,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -31028,7 +31028,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -31308,7 +31308,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -32148,7 +32148,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -36348,7 +36348,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -37472,7 +37472,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -38312,7 +38312,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -39992,7 +39992,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -41676,7 +41676,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -41956,7 +41956,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -42236,7 +42236,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -43076,7 +43076,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -44760,7 +44760,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -45596,7 +45596,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -45876,7 +45876,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -48676,7 +48676,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -48956,7 +48956,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -50636,7 +50636,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -50916,7 +50916,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -51196,7 +51196,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
@@ -51756,7 +51756,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -52316,7 +52316,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -52876,7 +52876,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -53156,7 +53156,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -53716,7 +53716,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -54276,7 +54276,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -54836,7 +54836,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
@@ -55116,7 +55116,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
@@ -55676,7 +55676,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -55956,7 +55956,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
@@ -58246,7 +58246,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -59374,7 +59374,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -61622,7 +61622,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">

</xml_diff>